<commit_message>
Update: checklist on external model integration completed
</commit_message>
<xml_diff>
--- a/co2routex/docs/pipeline_model_overview_v2.xlsx
+++ b/co2routex/docs/pipeline_model_overview_v2.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ykk/Documents/STORCITO/transport/co2routex/co2routex/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED0D520-7469-2740-A701-ED387B33CB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E0AE72C-48CE-744C-A68E-A63B9417DE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30220" yWindow="9040" windowWidth="38400" windowHeight="12560" activeTab="3" xr2:uid="{E8AD086B-54A1-F74B-9BE9-7CE5CD7C7DE9}"/>
+    <workbookView xWindow="0" yWindow="4260" windowWidth="30240" windowHeight="12560" xr2:uid="{E8AD086B-54A1-F74B-9BE9-7CE5CD7C7DE9}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="4" r:id="rId1"/>
     <sheet name="model_readiness_checklist" sheetId="3" r:id="rId2"/>
     <sheet name="model_attributes_overview" sheetId="1" r:id="rId3"/>
     <sheet name="data_sources" sheetId="2" r:id="rId4"/>
-    <sheet name="random_thoughts" sheetId="5" r:id="rId5"/>
+    <sheet name="external_integration_checklist" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="319">
   <si>
     <t>Programming</t>
   </si>
@@ -195,9 +195,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>EU-DEM</t>
-  </si>
-  <si>
     <t>25m</t>
   </si>
   <si>
@@ -228,9 +225,6 @@
     <t>EEA38</t>
   </si>
   <si>
-    <t>CDDA</t>
-  </si>
-  <si>
     <t>100m</t>
   </si>
   <si>
@@ -339,9 +333,6 @@
     <t>Metadata: https://ec.europa.eu/eurostat/cache/metadata/en/lan_esms.htm</t>
   </si>
   <si>
-    <t>LCM-10</t>
-  </si>
-  <si>
     <t>10m</t>
   </si>
   <si>
@@ -423,9 +414,6 @@
     <t>https://zenodo.org/records/14449495</t>
   </si>
   <si>
-    <t>gHMv3s</t>
-  </si>
-  <si>
     <t>gHMv3c</t>
   </si>
   <si>
@@ -462,36 +450,18 @@
     <t>1. Data collection &amp; standardisation</t>
   </si>
   <si>
-    <t>1. Data Collection &amp; Standardisation → 2. Preparatory Optimal Routing → 3. Mode-specific Constraints &amp; Parameterisation → 4. Cost Model Development → 5. Validation, Sensitivity &amp; Uncertainty → 6. Documentation &amp; Reproducibility</t>
-  </si>
-  <si>
-    <t>2. Preparatory Optimal Routing</t>
-  </si>
-  <si>
     <t>All major nodes (sources/sinks/utilisers) and existing infrastructure mapped with consistent quality.</t>
   </si>
   <si>
     <t>Feasible routing options and the associated distances pre-identified for all node pairs.</t>
   </si>
   <si>
-    <t>3. Mode-specific Constraints &amp; Parameterisation</t>
-  </si>
-  <si>
-    <t>Parameter tables and standardised database or GIS files.</t>
-  </si>
-  <si>
     <t>Standardised database or GIS files.</t>
   </si>
   <si>
     <t>All mode-specific technical and non-technical constraints and concerns fully defined and indexed.</t>
   </si>
   <si>
-    <t>4. Cost Model Development</t>
-  </si>
-  <si>
-    <t>Initial optimal routing scenarios and model to account for the associated matrices (e.g. distance, number of bends).</t>
-  </si>
-  <si>
     <t>Mode-specific cost model with embedded mathematical cost functions.</t>
   </si>
   <si>
@@ -507,9 +477,6 @@
     <t>Model behaviour confirmed and uncertainties characterised.</t>
   </si>
   <si>
-    <t>Parameterisation on mode-specific constraints and costs can also be tweaked by uncertainties in environmental or societal concerns.</t>
-  </si>
-  <si>
     <t>6. Documentation &amp; Reproducibility</t>
   </si>
   <si>
@@ -603,9 +570,6 @@
     <t>1a. CO₂ sources, sinks, utilisers: locations, flow rates and purity levels.                                              1b. Existing infrastructure: pipelines, rail/truck networks, ports, railway stations.</t>
   </si>
   <si>
-    <t>2a. Preliminary route identification (optimal connections) and network pre-processing (e.g. clustering of adjacent nodes).                               2b. Candidate arcs, distance matrices, potential transport switch nodes (according to intersection of candidate arcs).</t>
-  </si>
-  <si>
     <t>Intersections of candidate arcs may generate new potential transport switches, leading to additional node pairs and candidate arcs.</t>
   </si>
   <si>
@@ -756,24 +720,6 @@
     <t>File Name: pipeline_model_overview_v2.xlsx</t>
   </si>
   <si>
-    <t>Routing (find the path and the associated distance).</t>
-  </si>
-  <si>
-    <t>transport model components</t>
-  </si>
-  <si>
-    <t>gridded friction/resistance map &lt;- parameterise the factors</t>
-  </si>
-  <si>
-    <t>clustering method</t>
-  </si>
-  <si>
-    <t>how to connect method</t>
-  </si>
-  <si>
-    <t>HWSDv2.0</t>
-  </si>
-  <si>
     <t>Food and Agriculture Organization of the United Nations</t>
   </si>
   <si>
@@ -810,21 +756,12 @@
     <t>https://metadata.europe-geology.eu/record/basic/5f7db57f-6e84-4484-835f-706b0a010833</t>
   </si>
   <si>
-    <t>10000m</t>
-  </si>
-  <si>
     <t>² Shapefile (SHP) and GeoPackage (GPKG) are widely supported in both open-source environments (e.g. Python) and GIS tools (e.g. ArcGIS), while Geodatabase (GDB) is primarily processed with GIS tools. Microsoft Access Database (MDB) is a tabular database format rather than a native GIS layer format and is typically used for attribute storage or converted for analysis.</t>
   </si>
   <si>
-    <t>GLiM⁴</t>
-  </si>
-  <si>
     <t>ArcGIS⁵</t>
   </si>
   <si>
-    <t>EDGI1:1M⁶</t>
-  </si>
-  <si>
     <t>Seismic risk⁷</t>
   </si>
   <si>
@@ -846,9 +783,6 @@
     <t>⁸ The esrm20 dataset has a spatial resolution of 0.1∘ × 0.1∘ means the raster pixels will be rectangular, not perfectly square. Every pixel will be around 11100m tall, but the width will steadly shrink from about 9100m at the bottom of the map down to 3800m at the very top.</t>
   </si>
   <si>
-    <t>1000m⁸</t>
-  </si>
-  <si>
     <t>N/A⁹</t>
   </si>
   <si>
@@ -882,9 +816,6 @@
     <t>⁹ The underlying historical and instrumental data used to build the model spans from the year 1000 to December 31, 2014. However the final raster maps are time-independent probabilistic forecasts. They represent the probability of ground shaking exceedance over a 50-year time span for specific mean return periods (50, 475, 975, 2500, and 5000 years).</t>
   </si>
   <si>
-    <t>Last Updated: 19th April 2026</t>
-  </si>
-  <si>
     <t>CO₂ Pipeline Network Optimisation Model: Overview, Workflow, Data Source &amp; Documentation</t>
   </si>
   <si>
@@ -894,9 +825,6 @@
     <t>¹⁰ The GEM dataset represents a 50-year future projection of seismic risk, it is grounded in historical and instrumental data spanning from 1904 to 2021, with supplementary historical data extending back over a millennium.</t>
   </si>
   <si>
-    <t>GEM-GHSM</t>
-  </si>
-  <si>
     <t>N/A¹¹</t>
   </si>
   <si>
@@ -906,26 +834,176 @@
     <t>¹² The CDDA dataset is a vector dataset with no fixed pixel size; however, its scale of 1:100,000 corresponds approximately to an effective spatial resolution of ~1000 m, meaning features smaller than this are generally not reliably represented.</t>
   </si>
   <si>
-    <t>10000m¹²</t>
-  </si>
-  <si>
     <t>¹³ The JRC-ESTAT Census Population Grid 2021 was derived from the CENSUS 2021 1km grid as a collaboration between JRC and Eurostat.</t>
   </si>
   <si>
-    <t>JRC-ESTAT Census Population Grid 2021¹³</t>
-  </si>
-  <si>
     <t>¹⁴  The GHS-POP-R2023A was derived from GPWv4, which offers higher-resolution gridded data (100m) along with projections for 2025 and 2030.</t>
   </si>
   <si>
     <t>GHS-POP-R2023A¹⁴</t>
+  </si>
+  <si>
+    <t>2a. Preliminary route identification (feasible connections) and network pre-processing (e.g. clustering of adjacent nodes).                               2b. Candidate arcs, distance matrices, potential transport switch nodes (according to intersection of candidate arcs).</t>
+  </si>
+  <si>
+    <t>Initial feasible routing scenarios and model to provide with potential transport switches, and account for the associated matrices (e.g. distance, number of bends).</t>
+  </si>
+  <si>
+    <t>Parameter tables, standardised database or GIS files.</t>
+  </si>
+  <si>
+    <t>2. Mode-specific Constraints &amp; Parameterisation</t>
+  </si>
+  <si>
+    <t>Parameterisation on mode-specific constraints and costs can also be tweaked to account for uncertainties related to environmental or societal concerns, in line with user demand.</t>
+  </si>
+  <si>
+    <t>[EU-DEM]</t>
+  </si>
+  <si>
+    <t>[LCM-10]</t>
+  </si>
+  <si>
+    <t>[HWSDv2.0]</t>
+  </si>
+  <si>
+    <t>[GLiM⁴]</t>
+  </si>
+  <si>
+    <t>10000m⁸</t>
+  </si>
+  <si>
+    <t>[GEM-GHSM]</t>
+  </si>
+  <si>
+    <t>1000m¹²</t>
+  </si>
+  <si>
+    <t>EDGI1:1M</t>
+  </si>
+  <si>
+    <t>10000m⁶</t>
+  </si>
+  <si>
+    <t>[OSM]</t>
+  </si>
+  <si>
+    <t>[CDDA]</t>
+  </si>
+  <si>
+    <t>[gHMv3s]</t>
+  </si>
+  <si>
+    <t>[JRC-ESTAT Census Population Grid 2021]¹³</t>
+  </si>
+  <si>
+    <t>Datasets whose names are enclosed in [ ] are those selected for subsequent parameterisation steps. If more than one dataset is enclosed in [ ] within the same category, this indicates that multiple candidates are provisionally suitable and require further in-depth comparison (e.g., one may offer higher spatial resolution while another provides more up-to-date data).</t>
+  </si>
+  <si>
+    <t>3. Cost Model Development</t>
+  </si>
+  <si>
+    <t>4. Preparatory Optimal Routing</t>
+  </si>
+  <si>
+    <t>1. Data Collection &amp; Standardisation → 2. Mode-specific Constraints &amp; Parameterisation → 3. Cost Model Development → 4. Preparatory Optimal Routin → 5. Validation, Sensitivity &amp; Uncertainty → 6. Documentation &amp; Reproducibility</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>co2routex v1.0 Scope &amp; Status</t>
+  </si>
+  <si>
+    <t>co2routex v2.0 Scope &amp; Status</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>Script</t>
+  </si>
+  <si>
+    <t>Mode-specific constraint parameters</t>
+  </si>
+  <si>
+    <t>Existing CO₂ transport networks</t>
+  </si>
+  <si>
+    <t>Potential transport switches</t>
+  </si>
+  <si>
+    <t>Mode-specific cost formulations</t>
+  </si>
+  <si>
+    <t>Feasible node connection algorithms</t>
+  </si>
+  <si>
+    <t>Node clustering algorithms</t>
+  </si>
+  <si>
+    <t>Routing algorithms</t>
+  </si>
+  <si>
+    <t>Scenario analysis data</t>
+  </si>
+  <si>
+    <t>Gridded map data containing parameters for mode-specific transport constraints.</t>
+  </si>
+  <si>
+    <t>Data mapping current, mode-specific CO2 transport infrastructure.</t>
+  </si>
+  <si>
+    <t>Known switch nodes across modes (e.g., ports, railway stations, neutral intersections of road components).</t>
+  </si>
+  <si>
+    <t>Formulations to calculate transport costs depending on the chosen mode.</t>
+  </si>
+  <si>
+    <t>Algorithms to determine viable connections between nodes based on the transport mode.</t>
+  </si>
+  <si>
+    <t>Algorithms designed to cluster spatial nodes for optimized transport modeling.</t>
+  </si>
+  <si>
+    <t>Core algorithms for determining optimal transport routes.</t>
+  </si>
+  <si>
+    <t>Gridded map data for external risks and contingencies (e.g., seismic risks, backup transport routes).</t>
+  </si>
+  <si>
+    <t>Case study countries</t>
+  </si>
+  <si>
+    <t>Tested&amp; validated with dummy data</t>
+  </si>
+  <si>
+    <t>Not Applicable</t>
+  </si>
+  <si>
+    <t>Included</t>
+  </si>
+  <si>
+    <t>Pan-European</t>
+  </si>
+  <si>
+    <t>Tested &amp; validated with real-world nodes (case study countries)</t>
+  </si>
+  <si>
+    <t>Last Updated: 22nd April 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -981,16 +1059,35 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="38">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -1461,11 +1558,56 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1601,6 +1743,15 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1625,33 +1776,50 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1994,27 +2162,27 @@
   <sheetData>
     <row r="2" spans="2:2" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="32" t="s">
-        <v>281</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
-        <v>280</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -2038,31 +2206,31 @@
   <sheetData>
     <row r="2" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="32" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
-        <v>140</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="32" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="28" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="E6" s="30" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F6" s="31" t="s">
         <v>50</v>
@@ -2070,104 +2238,104 @@
     </row>
     <row r="7" spans="2:6" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="73" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="25" t="s">
+        <v>270</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="D8" s="69" t="s">
+        <v>269</v>
+      </c>
+      <c r="E8" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="C7" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>146</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="F7" s="21" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" ht="90" x14ac:dyDescent="0.2">
-      <c r="B8" s="26" t="s">
+      <c r="F8" s="21" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="73" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="26" t="s">
+        <v>286</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9" s="13" t="s">
         <v>141</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>187</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" ht="75" x14ac:dyDescent="0.2">
-      <c r="B9" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>147</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="10" spans="2:6" ht="71" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:6" ht="90" x14ac:dyDescent="0.2">
       <c r="B10" s="26" t="s">
-        <v>148</v>
+        <v>287</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>200</v>
+        <v>267</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>150</v>
+        <v>268</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" ht="90" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="89" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="26" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>155</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="61" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B12" s="27" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.2">
@@ -2199,25 +2367,25 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B3" s="62" t="s">
+      <c r="B3" s="68" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B4" s="62"/>
+      <c r="B4" s="68"/>
       <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
@@ -2226,16 +2394,16 @@
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B5" s="62"/>
+      <c r="B5" s="68"/>
       <c r="C5" s="1" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="68" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -2246,34 +2414,34 @@
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B7" s="62"/>
+      <c r="B7" s="68"/>
       <c r="C7" s="1" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B8" s="62"/>
+      <c r="B8" s="68"/>
       <c r="C8" s="1" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B9" s="62"/>
+      <c r="B9" s="68"/>
       <c r="C9" s="1" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B10" s="62" t="s">
+      <c r="B10" s="68" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -2284,7 +2452,7 @@
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B11" s="62"/>
+      <c r="B11" s="68"/>
       <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
@@ -2293,36 +2461,36 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="62" t="s">
+      <c r="B12" s="68" t="s">
         <v>15</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D12" s="51" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B13" s="62"/>
+      <c r="B13" s="68"/>
       <c r="C13" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B14" s="62"/>
+      <c r="B14" s="68"/>
       <c r="C14" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D14" s="51" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="62" t="s">
+      <c r="B15" s="68" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -2333,7 +2501,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B16" s="62"/>
+      <c r="B16" s="68"/>
       <c r="C16" s="1" t="s">
         <v>4</v>
       </c>
@@ -2342,108 +2510,108 @@
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="62"/>
+      <c r="B17" s="68"/>
       <c r="C17" s="1" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B18" s="62"/>
+      <c r="B18" s="68"/>
       <c r="C18" s="1" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B19" s="62"/>
+      <c r="B19" s="68"/>
       <c r="C19" s="1" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="62" t="s">
+      <c r="B20" s="68" t="s">
         <v>12</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B21" s="62"/>
+      <c r="B21" s="68"/>
       <c r="C21" s="1" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B22" s="62"/>
+      <c r="B22" s="68"/>
       <c r="C22" s="1" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B23" s="62"/>
+      <c r="B23" s="68"/>
       <c r="C23" s="1" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B24" s="62" t="s">
+      <c r="B24" s="68" t="s">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B25" s="62"/>
+      <c r="B25" s="68"/>
       <c r="C25" s="1" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B26" s="61" t="s">
-        <v>221</v>
+      <c r="B26" s="67" t="s">
+        <v>209</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B27" s="61"/>
+      <c r="B27" s="67"/>
       <c r="C27" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.2">
@@ -2451,37 +2619,37 @@
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B30" s="1" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B32" s="1" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B33" s="1" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B34" s="1" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -2502,7 +2670,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAC7E1D8-D6E4-2E4C-AB1F-BC7A2F73FD97}">
-  <dimension ref="B1:O42"/>
+  <dimension ref="B1:O44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="5" customWidth="1"/>
@@ -2511,7 +2679,7 @@
     <col min="4" max="4" width="29.33203125" style="5" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" style="5" customWidth="1"/>
     <col min="6" max="6" width="10.1640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="35.33203125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="43.33203125" style="5" customWidth="1"/>
     <col min="8" max="8" width="9" style="5" customWidth="1"/>
     <col min="9" max="9" width="11.1640625" style="5" customWidth="1"/>
     <col min="10" max="10" width="4" style="5" customWidth="1"/>
@@ -2545,13 +2713,13 @@
         <v>45</v>
       </c>
       <c r="I2" s="46" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J2" s="46" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K2" s="46" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L2" s="46" t="s">
         <v>47</v>
@@ -2567,1099 +2735,1106 @@
       </c>
     </row>
     <row r="3" spans="2:15" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="61" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="50" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>51</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>52</v>
       </c>
       <c r="G3" s="11">
         <v>2011</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="K3" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L3" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="L3" s="11" t="s">
-        <v>58</v>
-      </c>
       <c r="M3" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="N3" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="N3" s="11" t="s">
-        <v>56</v>
-      </c>
       <c r="O3" s="38" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B4" s="59"/>
+      <c r="B4" s="62"/>
       <c r="C4" s="50" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>51</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>52</v>
       </c>
       <c r="G4" s="11">
         <v>2011</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I4" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B5" s="62"/>
+      <c r="C5" s="56" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="J5" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="K5" s="36" t="s">
+        <v>98</v>
+      </c>
+      <c r="L5" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="M5" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="N5" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="O5" s="39" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B6" s="62"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="G6" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="H6" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J6" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="L6" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="N6" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="O6" s="40" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B7" s="62"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="K4" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="M4" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="O4" s="38" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B5" s="59"/>
-      <c r="C5" s="53" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" s="36" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="G5" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="I5" s="36" t="s">
-        <v>72</v>
-      </c>
-      <c r="J5" s="33" t="s">
-        <v>73</v>
-      </c>
-      <c r="K5" s="36" t="s">
-        <v>101</v>
-      </c>
-      <c r="L5" s="33" t="s">
-        <v>64</v>
-      </c>
-      <c r="M5" s="36" t="s">
-        <v>68</v>
-      </c>
-      <c r="N5" s="33" t="s">
-        <v>69</v>
-      </c>
-      <c r="O5" s="39" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B6" s="59"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="F6" s="34" t="s">
+      <c r="E7" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="G6" s="34" t="s">
+      <c r="F7" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="G7" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="H7" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J7" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="J6" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="L6" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="M6" s="5" t="s">
+      <c r="L7" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="N7" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="O7" s="40" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B8" s="62"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="F8" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="H8" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="J8" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="N6" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="O6" s="40" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B7" s="59"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="E7" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="F7" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="G7" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="H7" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="J7" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="L7" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="N7" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="O7" s="40" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B8" s="59"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="F8" s="34" t="s">
+      <c r="K8" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="G8" s="34" t="s">
+      <c r="L8" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="N8" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="H8" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="J8" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="K8" s="5" t="s">
+      <c r="O8" s="40" t="s">
         <v>96</v>
       </c>
-      <c r="L8" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="N8" s="34" t="s">
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B9" s="62"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="34" t="s">
         <v>97</v>
-      </c>
-      <c r="O8" s="40" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B9" s="59"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="E9" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="F9" s="34" t="s">
-        <v>100</v>
       </c>
       <c r="G9" s="34">
         <v>2020</v>
       </c>
       <c r="H9" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I9" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="L9" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="N9" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="O9" s="40" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B10" s="62"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="F10" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="H10" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="J10" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="L10" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="N10" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="O10" s="40" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B11" s="62"/>
+      <c r="C11" s="58"/>
+      <c r="D11" s="37" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="L9" s="34" t="s">
+      <c r="G11" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="H11" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="I11" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="J11" s="35" t="s">
+        <v>78</v>
+      </c>
+      <c r="K11" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="M9" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="N9" s="34" t="s">
-        <v>102</v>
-      </c>
-      <c r="O9" s="40" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B10" s="59"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="E10" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="F10" s="34" t="s">
-        <v>105</v>
-      </c>
-      <c r="G10" s="34" t="s">
-        <v>106</v>
-      </c>
-      <c r="H10" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="J10" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="L10" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="M10" s="5" t="s">
+      <c r="L11" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="M11" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="N11" s="35" t="s">
+        <v>113</v>
+      </c>
+      <c r="O11" s="41" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B12" s="62"/>
+      <c r="C12" s="56" t="s">
+        <v>200</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E12" s="55" t="s">
+        <v>154</v>
+      </c>
+      <c r="F12" s="55" t="s">
+        <v>149</v>
+      </c>
+      <c r="G12" s="55">
+        <v>2006</v>
+      </c>
+      <c r="H12" s="55" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="J12" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="K12" s="55" t="s">
+        <v>204</v>
+      </c>
+      <c r="L12" s="53" t="s">
+        <v>205</v>
+      </c>
+      <c r="M12" s="55" t="s">
+        <v>207</v>
+      </c>
+      <c r="N12" s="55" t="s">
+        <v>206</v>
+      </c>
+      <c r="O12" s="39" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B13" s="62"/>
+      <c r="C13" s="64"/>
+      <c r="D13" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="E13" s="53" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="53" t="s">
+        <v>149</v>
+      </c>
+      <c r="G13" s="53">
+        <v>2023</v>
+      </c>
+      <c r="H13" s="53" t="s">
+        <v>52</v>
+      </c>
+      <c r="I13" s="34" t="s">
+        <v>228</v>
+      </c>
+      <c r="J13" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K13" s="53" t="s">
+        <v>226</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="M13" s="53" t="s">
         <v>108</v>
       </c>
-      <c r="N10" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="O10" s="40" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B11" s="59"/>
-      <c r="C11" s="55"/>
-      <c r="D11" s="37" t="s">
-        <v>114</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="35" t="s">
+      <c r="N13" s="53" t="s">
+        <v>227</v>
+      </c>
+      <c r="O13" s="53" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B14" s="62"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="E14" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="G11" s="35" t="s">
-        <v>113</v>
-      </c>
-      <c r="H11" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="I11" s="37" t="s">
-        <v>72</v>
-      </c>
-      <c r="J11" s="35" t="s">
-        <v>80</v>
-      </c>
-      <c r="K11" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="L11" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="M11" s="37" t="s">
+      <c r="F14" s="53" t="s">
+        <v>229</v>
+      </c>
+      <c r="G14" s="53">
+        <v>2013</v>
+      </c>
+      <c r="H14" s="53" t="s">
         <v>115</v>
       </c>
-      <c r="N11" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="O11" s="41" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B12" s="59"/>
-      <c r="C12" s="53" t="s">
-        <v>212</v>
-      </c>
-      <c r="D12" s="66" t="s">
-        <v>215</v>
-      </c>
-      <c r="E12" s="69" t="s">
-        <v>165</v>
-      </c>
-      <c r="F12" s="69" t="s">
-        <v>160</v>
-      </c>
-      <c r="G12" s="69">
-        <v>2006</v>
-      </c>
-      <c r="H12" s="69" t="s">
-        <v>118</v>
-      </c>
-      <c r="I12" s="33" t="s">
-        <v>72</v>
-      </c>
-      <c r="J12" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="K12" s="69" t="s">
-        <v>216</v>
-      </c>
-      <c r="L12" s="67" t="s">
-        <v>217</v>
-      </c>
-      <c r="M12" s="69" t="s">
-        <v>219</v>
-      </c>
-      <c r="N12" s="69" t="s">
-        <v>218</v>
-      </c>
-      <c r="O12" s="39" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B13" s="59"/>
-      <c r="C13" s="65"/>
-      <c r="D13" s="66" t="s">
-        <v>243</v>
-      </c>
-      <c r="E13" s="67" t="s">
-        <v>76</v>
-      </c>
-      <c r="F13" s="67" t="s">
-        <v>160</v>
-      </c>
-      <c r="G13" s="67">
-        <v>2023</v>
-      </c>
-      <c r="H13" s="67" t="s">
-        <v>53</v>
-      </c>
-      <c r="I13" s="34" t="s">
-        <v>246</v>
-      </c>
-      <c r="J13" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="K13" s="67" t="s">
-        <v>244</v>
-      </c>
-      <c r="L13" s="66" t="s">
-        <v>64</v>
-      </c>
-      <c r="M13" s="67" t="s">
-        <v>111</v>
-      </c>
-      <c r="N13" s="67" t="s">
+      <c r="I14" s="34" t="s">
+        <v>239</v>
+      </c>
+      <c r="J14" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K14" s="53" t="s">
+        <v>230</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="M14" s="53" t="s">
+        <v>233</v>
+      </c>
+      <c r="N14" s="53" t="s">
+        <v>232</v>
+      </c>
+      <c r="O14" s="53" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B15" s="62"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="37" t="s">
+        <v>279</v>
+      </c>
+      <c r="E15" s="54" t="s">
+        <v>154</v>
+      </c>
+      <c r="F15" s="54" t="s">
+        <v>280</v>
+      </c>
+      <c r="G15" s="54">
+        <v>2016</v>
+      </c>
+      <c r="H15" s="54" t="s">
+        <v>115</v>
+      </c>
+      <c r="I15" s="35" t="s">
+        <v>235</v>
+      </c>
+      <c r="J15" s="35" t="s">
+        <v>78</v>
+      </c>
+      <c r="K15" s="54" t="s">
+        <v>234</v>
+      </c>
+      <c r="L15" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="M15" s="54" t="s">
+        <v>108</v>
+      </c>
+      <c r="N15" s="54" t="s">
+        <v>237</v>
+      </c>
+      <c r="O15" s="41" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B16" s="62"/>
+      <c r="C16" s="65" t="s">
+        <v>240</v>
+      </c>
+      <c r="D16" s="33" t="s">
         <v>245</v>
       </c>
-      <c r="O13" s="67" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B14" s="59"/>
-      <c r="C14" s="65"/>
-      <c r="D14" s="66" t="s">
-        <v>258</v>
-      </c>
-      <c r="E14" s="67" t="s">
-        <v>76</v>
-      </c>
-      <c r="F14" s="67" t="s">
+      <c r="E16" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="F16" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="G16" s="33" t="s">
         <v>247</v>
       </c>
-      <c r="G14" s="67">
-        <v>2013</v>
-      </c>
-      <c r="H14" s="67" t="s">
-        <v>118</v>
-      </c>
-      <c r="I14" s="34" t="s">
-        <v>259</v>
-      </c>
-      <c r="J14" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="K14" s="67" t="s">
+      <c r="H16" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="I16" s="36" t="s">
         <v>248</v>
       </c>
-      <c r="L14" s="66" t="s">
+      <c r="J16" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="K16" s="36" t="s">
+        <v>250</v>
+      </c>
+      <c r="L16" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="M16" s="33" t="s">
         <v>249</v>
       </c>
-      <c r="M14" s="67" t="s">
+      <c r="N16" s="33" t="s">
+        <v>252</v>
+      </c>
+      <c r="O16" s="39" t="s">
         <v>251</v>
-      </c>
-      <c r="N14" s="67" t="s">
-        <v>250</v>
-      </c>
-      <c r="O14" s="67" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B15" s="59"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="37" t="s">
-        <v>260</v>
-      </c>
-      <c r="E15" s="68" t="s">
-        <v>165</v>
-      </c>
-      <c r="F15" s="68" t="s">
-        <v>256</v>
-      </c>
-      <c r="G15" s="68">
-        <v>2016</v>
-      </c>
-      <c r="H15" s="68" t="s">
-        <v>118</v>
-      </c>
-      <c r="I15" s="35" t="s">
-        <v>253</v>
-      </c>
-      <c r="J15" s="35" t="s">
-        <v>80</v>
-      </c>
-      <c r="K15" s="68" t="s">
-        <v>252</v>
-      </c>
-      <c r="L15" s="68" t="s">
-        <v>64</v>
-      </c>
-      <c r="M15" s="68" t="s">
-        <v>111</v>
-      </c>
-      <c r="N15" s="68" t="s">
-        <v>255</v>
-      </c>
-      <c r="O15" s="41" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B16" s="59"/>
-      <c r="C16" s="63" t="s">
-        <v>261</v>
-      </c>
-      <c r="D16" s="33" t="s">
-        <v>266</v>
-      </c>
-      <c r="E16" s="33" t="s">
-        <v>165</v>
-      </c>
-      <c r="F16" s="33" t="s">
-        <v>268</v>
-      </c>
-      <c r="G16" s="33" t="s">
-        <v>269</v>
-      </c>
-      <c r="H16" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="I16" s="36" t="s">
-        <v>270</v>
-      </c>
-      <c r="J16" s="33" t="s">
-        <v>73</v>
-      </c>
-      <c r="K16" s="36" t="s">
-        <v>272</v>
-      </c>
-      <c r="L16" s="33" t="s">
-        <v>64</v>
-      </c>
-      <c r="M16" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="N16" s="33" t="s">
-        <v>274</v>
-      </c>
-      <c r="O16" s="39" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B17" s="52"/>
-      <c r="C17" s="64"/>
+      <c r="C17" s="66"/>
       <c r="D17" s="37" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="G17" s="35" t="s">
-        <v>282</v>
+        <v>259</v>
       </c>
       <c r="H17" s="35" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I17" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="K17" s="35" t="s">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="L17" s="35" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="M17" s="35" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="N17" s="35" t="s">
-        <v>276</v>
+        <v>254</v>
       </c>
       <c r="O17" s="41" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="2:15" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="61" t="s">
         <v>12</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>117</v>
+        <v>281</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>285</v>
+        <v>261</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="O18" s="38" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="59"/>
+      <c r="B19" s="62"/>
       <c r="C19" s="50" t="s">
         <v>5</v>
       </c>
       <c r="D19" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="J19" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L19" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>288</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="J19" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="K19" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="L19" s="11" t="s">
-        <v>64</v>
-      </c>
       <c r="M19" s="11" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="O19" s="38" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" spans="2:15" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="59"/>
-      <c r="C20" s="53" t="s">
+      <c r="B20" s="62"/>
+      <c r="C20" s="56" t="s">
         <v>1</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>127</v>
+        <v>283</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G20" s="33">
         <v>2022</v>
       </c>
       <c r="H20" s="36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I20" s="33" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J20" s="36" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="K20" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="L20" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="M20" s="33" t="s">
+        <v>120</v>
+      </c>
+      <c r="N20" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="O20" s="42" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="21" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="62"/>
+      <c r="C21" s="58"/>
+      <c r="D21" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="L20" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="M20" s="33" t="s">
+      <c r="E21" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="F21" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" s="35" t="s">
+        <v>118</v>
+      </c>
+      <c r="H21" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="I21" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="J21" s="37" t="s">
+        <v>78</v>
+      </c>
+      <c r="K21" s="35" t="s">
+        <v>121</v>
+      </c>
+      <c r="L21" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="M21" s="35" t="s">
+        <v>119</v>
+      </c>
+      <c r="N21" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="N20" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="O20" s="42" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="21" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="59"/>
-      <c r="C21" s="55"/>
-      <c r="D21" s="37" t="s">
-        <v>128</v>
-      </c>
-      <c r="E21" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="F21" s="37" t="s">
-        <v>105</v>
-      </c>
-      <c r="G21" s="35" t="s">
-        <v>121</v>
-      </c>
-      <c r="H21" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="I21" s="35" t="s">
-        <v>72</v>
-      </c>
-      <c r="J21" s="37" t="s">
-        <v>80</v>
-      </c>
-      <c r="K21" s="35" t="s">
-        <v>124</v>
-      </c>
-      <c r="L21" s="37" t="s">
-        <v>64</v>
-      </c>
-      <c r="M21" s="35" t="s">
-        <v>122</v>
-      </c>
-      <c r="N21" s="35" t="s">
-        <v>126</v>
-      </c>
       <c r="O21" s="43" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="22" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="59"/>
-      <c r="C22" s="56" t="s">
+      <c r="B22" s="62"/>
+      <c r="C22" s="59" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" s="33" t="s">
+        <v>149</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="H22" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J22" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="L22" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="M22" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="N22" s="33" t="s">
+        <v>152</v>
+      </c>
+      <c r="O22" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="23" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="62"/>
+      <c r="C23" s="59"/>
+      <c r="D23" s="34" t="s">
         <v>159</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F22" s="33" t="s">
+      <c r="E23" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="F23" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="H23" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="J23" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="L23" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="M23" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="N23" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="H22" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="I22" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="J22" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="K22" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="L22" s="33" t="s">
-        <v>64</v>
-      </c>
-      <c r="M22" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="N22" s="33" t="s">
-        <v>163</v>
-      </c>
-      <c r="O22" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="23" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="59"/>
-      <c r="C23" s="56"/>
-      <c r="D23" s="34" t="s">
-        <v>170</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="F23" s="34" t="s">
-        <v>160</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="H23" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="J23" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="K23" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="L23" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="M23" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="N23" s="34" t="s">
-        <v>171</v>
-      </c>
       <c r="O23" s="7" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="59"/>
-      <c r="C24" s="56"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="59"/>
       <c r="D24" s="34" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="F24" s="34" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G24" s="5">
         <v>2021</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J24" s="34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="L24" s="34" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="M24" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N24" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="25" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="62"/>
+      <c r="C25" s="59"/>
+      <c r="D25" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="H25" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J25" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="L25" s="34" t="s">
+        <v>163</v>
+      </c>
+      <c r="M25" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="N25" s="34" t="s">
+        <v>165</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="26" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="62"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F26" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H26" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J26" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K26" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="L26" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="M26" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="N26" s="34" t="s">
+        <v>168</v>
+      </c>
+      <c r="O26" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="N24" s="34" t="s">
-        <v>168</v>
-      </c>
-      <c r="O24" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="25" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="59"/>
-      <c r="C25" s="56"/>
-      <c r="D25" s="34" t="s">
+    </row>
+    <row r="27" spans="2:15" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="63"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="44" t="s">
+        <v>171</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="F27" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H27" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J27" s="44" t="s">
+        <v>78</v>
+      </c>
+      <c r="K27" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="L27" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="M27" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="N27" s="44" t="s">
         <v>172</v>
       </c>
-      <c r="E25" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F25" s="34" t="s">
-        <v>160</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="H25" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="J25" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="L25" s="34" t="s">
-        <v>174</v>
-      </c>
-      <c r="M25" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="N25" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="O25" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="26" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="59"/>
-      <c r="C26" s="56"/>
-      <c r="D26" s="34" t="s">
-        <v>292</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F26" s="34" t="s">
-        <v>180</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="H26" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="J26" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="L26" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="M26" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="N26" s="34" t="s">
-        <v>179</v>
-      </c>
-      <c r="O26" s="7" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="27" spans="2:15" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="60"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="44" t="s">
-        <v>182</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="F27" s="44" t="s">
-        <v>160</v>
-      </c>
-      <c r="G27" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="H27" s="44" t="s">
-        <v>53</v>
-      </c>
-      <c r="I27" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="J27" s="44" t="s">
-        <v>80</v>
-      </c>
-      <c r="K27" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="L27" s="44" t="s">
-        <v>64</v>
-      </c>
-      <c r="M27" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="N27" s="44" t="s">
-        <v>183</v>
-      </c>
       <c r="O27" s="10" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B29" s="5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B30" s="5" t="s">
-        <v>257</v>
+        <v>238</v>
       </c>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B31" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B32" s="5" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B33" s="5" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B34" s="5" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B35" s="5" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B36" s="5" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B37" s="5" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B38" s="5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B39" s="5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B40" s="5" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B41" s="5" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B33" s="5" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B34" s="5" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B35" s="5" t="s">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B42" s="5" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B36" s="5" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B37" s="5" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B38" s="5" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B39" s="5" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B40" s="5" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B41" s="5" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B42" s="5" t="s">
-        <v>291</v>
-      </c>
+    <row r="44" spans="2:3" ht="149" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B44" s="70" t="s">
+        <v>285</v>
+      </c>
+      <c r="C44" s="70"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="B44:C44"/>
     <mergeCell ref="C5:C11"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="C22:C27"/>
@@ -3675,32 +3850,196 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9212F2E9-CB06-8642-8120-D52F93788C70}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="B1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4.33203125" customWidth="1"/>
+    <col min="3" max="3" width="15.5" customWidth="1"/>
+    <col min="4" max="4" width="20.1640625" customWidth="1"/>
+    <col min="5" max="5" width="45.5" customWidth="1"/>
+    <col min="6" max="6" width="30.5" customWidth="1"/>
+    <col min="7" max="7" width="30.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>242</v>
+    <row r="1" spans="2:7" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" s="71" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="74" t="s">
+        <v>289</v>
+      </c>
+      <c r="C2" s="75" t="s">
+        <v>290</v>
+      </c>
+      <c r="D2" s="75" t="s">
+        <v>291</v>
+      </c>
+      <c r="E2" s="75" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="75" t="s">
+        <v>292</v>
+      </c>
+      <c r="G2" s="76" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="77">
+        <v>1</v>
+      </c>
+      <c r="C3" s="72" t="s">
+        <v>294</v>
+      </c>
+      <c r="D3" s="73" t="s">
+        <v>296</v>
+      </c>
+      <c r="E3" s="73" t="s">
+        <v>304</v>
+      </c>
+      <c r="F3" s="72" t="s">
+        <v>312</v>
+      </c>
+      <c r="G3" s="78" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="B4" s="77">
+        <v>2</v>
+      </c>
+      <c r="C4" s="72" t="s">
+        <v>294</v>
+      </c>
+      <c r="D4" s="73" t="s">
+        <v>297</v>
+      </c>
+      <c r="E4" s="73" t="s">
+        <v>305</v>
+      </c>
+      <c r="F4" s="72" t="s">
+        <v>312</v>
+      </c>
+      <c r="G4" s="78" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="77">
+        <v>3</v>
+      </c>
+      <c r="C5" s="72" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" s="73" t="s">
+        <v>298</v>
+      </c>
+      <c r="E5" s="73" t="s">
+        <v>306</v>
+      </c>
+      <c r="F5" s="73" t="s">
+        <v>312</v>
+      </c>
+      <c r="G5" s="79" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="77">
+        <v>4</v>
+      </c>
+      <c r="C6" s="72" t="s">
+        <v>295</v>
+      </c>
+      <c r="D6" s="73" t="s">
+        <v>299</v>
+      </c>
+      <c r="E6" s="73" t="s">
+        <v>307</v>
+      </c>
+      <c r="F6" s="73" t="s">
+        <v>313</v>
+      </c>
+      <c r="G6" s="79" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="77">
+        <v>5</v>
+      </c>
+      <c r="C7" s="72" t="s">
+        <v>295</v>
+      </c>
+      <c r="D7" s="73" t="s">
+        <v>300</v>
+      </c>
+      <c r="E7" s="73" t="s">
+        <v>308</v>
+      </c>
+      <c r="F7" s="72" t="s">
+        <v>313</v>
+      </c>
+      <c r="G7" s="79" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="B8" s="77">
+        <v>6</v>
+      </c>
+      <c r="C8" s="72" t="s">
+        <v>295</v>
+      </c>
+      <c r="D8" s="73" t="s">
+        <v>301</v>
+      </c>
+      <c r="E8" s="73" t="s">
+        <v>309</v>
+      </c>
+      <c r="F8" s="72" t="s">
+        <v>313</v>
+      </c>
+      <c r="G8" s="79" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="77">
+        <v>7</v>
+      </c>
+      <c r="C9" s="72" t="s">
+        <v>295</v>
+      </c>
+      <c r="D9" s="73" t="s">
+        <v>302</v>
+      </c>
+      <c r="E9" s="73" t="s">
+        <v>310</v>
+      </c>
+      <c r="F9" s="72" t="s">
+        <v>313</v>
+      </c>
+      <c r="G9" s="79" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="80">
+        <v>8</v>
+      </c>
+      <c r="C10" s="81" t="s">
+        <v>294</v>
+      </c>
+      <c r="D10" s="82" t="s">
+        <v>303</v>
+      </c>
+      <c r="E10" s="82" t="s">
+        <v>311</v>
+      </c>
+      <c r="F10" s="81" t="s">
+        <v>314</v>
+      </c>
+      <c r="G10" s="83" t="s">
+        <v>315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>